<commit_message>
force main: prendi le mie modifiche locali
</commit_message>
<xml_diff>
--- a/resources/datapool_prova.xlsx
+++ b/resources/datapool_prova.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://clariter-my.sharepoint.com/personal/leonardo_diamanti_claritergroup_com/Documents/Desktop/Automation_silk/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="11_F25DC773A252ABDACC104895C19E7EF25ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7FC6F5F-7936-480A-B21D-BAD5E77BD224}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="11_F25DC773A252ABDACC104895C19E7EF25ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F776D923-4FCD-48D5-8CA1-C4088B899408}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="old" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="146">
   <si>
     <t>S0019.4.1.1</t>
   </si>
@@ -851,11 +851,20 @@
     <t>S001 prova</t>
   </si>
   <si>
-    <t>ciao - 9.1.1.1 Contenuti non testuali - S001 Prova:: (#D000… descrizione)</t>
-  </si>
-  <si>
-    <t>ciao - 9.4.1.2 Nome, ruolo, valore - S001 Prova:: (#D0023)
-02 Prova:: (#D000… descrizione)</t>
+    <t>S001 homepage</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.1.1.1 Contenuti non testuali - S001 homepage:</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.4.1.2 Contenuti non testuali - S002 homepage:</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.1.1.1 Contenuti non testuali - S001 homepage:: (#D000… descrizione)</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.4.1.2 Nome, ruolo, valore - S001 homepage:: (#D0023)
+02 homepage:: (#D000… descrizione)</t>
   </si>
 </sst>
 </file>
@@ -2247,6 +2256,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D33EDF36-8C7D-492E-9FD7-BEF33BB23ADC}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="75.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -2285,16 +2299,16 @@
         <v>132</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>36</v>
@@ -2312,16 +2326,16 @@
         <v>136</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
feat: MT flow + 9.6 rule; POM & config updates
</commit_message>
<xml_diff>
--- a/resources/datapool_prova.xlsx
+++ b/resources/datapool_prova.xlsx
@@ -8,26 +8,40 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://clariter-my.sharepoint.com/personal/leonardo_diamanti_claritergroup_com/Documents/Desktop/Automation_silk/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_F25DC773A252ABDACC104895C19E7EF25ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F776D923-4FCD-48D5-8CA1-C4088B899408}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="11_F25DC773A252ABDACC104895C19E7EF25ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9A50785-EE7E-4AAA-8AC8-9214EF871FBC}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="old" sheetId="1" r:id="rId1"/>
     <sheet name="Foglio" sheetId="2" r:id="rId2"/>
     <sheet name="Foglio1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="172">
   <si>
     <t>S0019.4.1.1</t>
   </si>
@@ -791,23 +805,109 @@
     <t>S0019.1.1.1</t>
   </si>
   <si>
-    <t>ciao - 9.1.1.1 Contenuti non testuali - S001 Prova:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ciao - 9.1.1.1 Contenuti non testuali - S001 Prova:: (#D0001)_x000D_
-S001 Prova_x000D_
-Requisito WCAG: 1.1.1_x000D_
-Disabilità afflitte: Blind;Deafblind_x000D_
+    <t>AP-00828</t>
+  </si>
+  <si>
+    <t>S0019.4.1.2</t>
+  </si>
+  <si>
+    <t>..SITO_RUO_SERVIZIPERTE_202509 ** FARE SETUP SILK AP/PK - INBOX - SERVIZI / EP **</t>
+  </si>
+  <si>
+    <t>S001 homepage</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.1.1.1 Contenuti non testuali - S001 homepage:</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.4.1.2 Contenuti non testuali - S002 homepage:</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.1.1.1 Contenuti non testuali - S001 homepage:: (#D000… descrizione)</t>
+  </si>
+  <si>
+    <t>serviziPerTe - 9.4.1.2 Nome, ruolo, valore - S001 homepage:: (#D0023)
+02 homepage:: (#D000… descrizione)</t>
+  </si>
+  <si>
+    <t>S0019.1.3.1</t>
+  </si>
+  <si>
+    <t>S0019.1.4.3</t>
+  </si>
+  <si>
+    <t>S0019.2.1.1</t>
+  </si>
+  <si>
+    <t>S0019.2.4.2</t>
+  </si>
+  <si>
+    <t>S0019.3.1.2</t>
+  </si>
+  <si>
+    <t>S0029.1.4.3</t>
+  </si>
+  <si>
+    <t>S0029.2.1.1</t>
+  </si>
+  <si>
+    <t>S0029.2.4.2</t>
+  </si>
+  <si>
+    <t>S0029.3.1.1</t>
+  </si>
+  <si>
+    <t>S0029.4.1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.1.3.1 Informazioni e correlazioni - S001 Raccolta Idee e Contributi:: (#TM0007)_x000D_
+S001 Raccolta Idee e Contributi_x000D_
+Requisito WCAG: 1.3.1_x000D_
+Disabilità afflitte: Blind;Deafblind;Low Vision;Mobility_x000D_
 Impatto Utente: 1 - Critical_x000D_
 _x000D_
 Descrizione_x000D_
-001 - Gli elementi immagine non hanno attributi '[alt]' - Gli elementi informativi dovrebbero mirare a un testo alternativo breve e descrittivo. Gli elementi decorativi possono essere ignorati con un attributo alt vuoto. [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.10/image-alt)_x000D_
+001 - Agli elementi form non sono associate etichette - Le etichette assicurano che i controlli delle form vengano annunciati correttamente dalle tecnologie assistive, come gli screen reader. [Ulteriori informazioni] (https://web.dev/label/)_x000D_
 _x000D_
 Esempio di violazione individuata sull'oggetto:_x000D_
-001 - https://posteitaliane.sharepoint.com/sites/NoiDiPoste-Collaudo/SitePages/PosteperTe/Servizi%20per%20la%20persona/Amministrazione/Servizi-amministrativi.aspx &lt;img src=\"/sites/NoiDiPoste-Collaudo/SiteAssets/Servizi%20per%20la%20persona/Icone/Aâ€¦\" class=\"classForImage_3a0fec79\"&gt; con selettore div#Presenze e assenze - Pianificazione presenze e assenze &gt; div.topBorderColor_3a0fec79 &gt; div.divForImage_3a0fec79 &gt; img.classForImage_3a0fec79_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;textarea appmagic-control="TextInput2_2textarea" class="appmagic-textarea mousetrap block-undo-redo" data-control-part="text" data-bind="
+      value: text,
+      css: {
+        underline: properties.Underline,
+        strikethrough: properties.Strikethrough,
+        readonly: viewState.displayMode() === AppMagic.Constants.DisplayMode.View
+      },
+      event: {
+        click: handleClick,
+        change: handleOnChange
+      },
+      attr: {
+        title: properties.Tooltip() || null,
+        'aria-label': properties.AccessibleLabel() || null,
+        placeholder: properties.HintText,
+        readonly: viewState.displayMode() === AppMagic.Constants.DisplayMode.View,
+        maxlength: properties.MaxLength() &amp;lt; 0 ? 0 : properties.MaxLength()
+      },
+      style: {
+        fontFamily: properties.Font,
+        fontSize: properties.Size,
+        color: autoProperties.Color,
+        fontWeight: properties.FontWeight,
+        fontStyle: properties.Italic,
+        textAlign: properties.Align,
+        lineHeight: properties.LineHeight,
+        paddingTop: properties.PaddingTop,
+        paddingRight: properties.PaddingRight,
+        paddingBottom: properties.PaddingBottom,
+        paddingLeft: properties.PaddingLeft
+      },
+      disable: viewState.displayMode() === AppMagic.Constants.DisplayMode.Disabled" placeholder="" disabled="" tabindex="370" style="font-family: &amp;quot;Open Sans&amp;quot;, sans-serif; font-size: 13pt; color: rgb(0, 0, 0); font-weight: normal; font-style: normal; text-align: left; line-height: 1.2; padding: 5px;"&gt; con selettore ["#fullscreen-app-host","textarea[appmagic-control=\"TextInput2_2textarea\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/88496147-9aed-4626-b4c4-7c2a7bafa246_x000D_
 _x000D_
 Possibile Metodologia Risolutiva:_x000D_
-001 - Fornisci un attributo alt descrittivo per ogni immagine. Questo consente agli screen reader di descrivere l’immagine agli utenti con disabilità visive, migliorando l’accessibilità del contenuto visivo._x000D_
+001 - Ogni campo del form dovrebbe avere un’etichetta associata tramite il tag &lt;label&gt; per facilitare l’interazione degli utenti che utilizzano tecnologie assistive. Le etichette devono descrivere chiaramente la funzione del campo._x000D_
 _x000D_
 Occorrenze rilevate: 1_x000D_
 _x000D_
@@ -815,29 +915,32 @@
 </t>
   </si>
   <si>
-    <t>AP-00828</t>
-  </si>
-  <si>
-    <t>S0019.4.1.2</t>
-  </si>
-  <si>
-    <t>ciao - 9.4.1.2 Contenuti non testuali - S002 Prova:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ciao - 9.4.1.2 Nome, ruolo, valore - S001 Prova:: (#D0023)_x000D_
-S001 Prova_x000D_
-Requisito WCAG: 4.1.2_x000D_
-Disabilità afflitte: Blind;Deafblind_x000D_
-Impatto Utente: 1 - Critical_x000D_
+    <t xml:space="preserve">RUO - Insieme - 9.1.4.3 Contrasto (minimo) - S001 Raccolta Idee e Contributi:: (#TM0018)_x000D_
+S001 Raccolta Idee e Contributi_x000D_
+Requisito WCAG: 1.4.3_x000D_
+Disabilità afflitte: Colorblindness;Low Vision_x000D_
+Impatto Utente: 2 - Serious_x000D_
 _x000D_
 Descrizione_x000D_
-001 - I pulsanti non hanno un nome accessibile - Quando un pulsante non ha un nome accessibile, le utilità per la lettura dello schermo lo annunciano come "pulsante", rendendolo inutilizzabile per gli utenti che si affidano alle utilità per la lettura dello schermo. [Ulteriori informazioni] (https://web.dev/button-name/)_x000D_
+001 - I colori di sfondo e di primo piano non hanno un rapporto di contrasto sufficiente. - Il testo a basso contrasto è difficile o impossibile da leggere per molti utenti. [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.10/color-contrast)_x000D_
 _x000D_
 Esempio di violazione individuata sull'oggetto:_x000D_
-001 - https://posteitaliane.sharepoint.com/sites/NoiDiPoste-Collaudo/SitePages/PosteperTe/Servizi%20per%20la%20persona/Amministrazione/Servizi-amministrativi.aspx &lt;button type=\"button\" role=\"menuitem\" class=\"ms-Button ms-Button--commandBar ms-Button--hasMenu ms-CommandBar-overflowBâ€¦\" data-is-focusable=\"true\" aria-expanded=\"false\" aria-haspopup=\"true\" tabindex=\"0\"&gt; con selettore div.ms-FocusZone &gt; div.ms-OverflowSet &gt; div.ms-OverflowSet-overflowButton &gt; button.ms-Button_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div spellcheck="false" unselectable="off" class="appmagic-label-text" data-control-part="text" data-bind="{
+            inlineEditText: properties.Text,
+            css: {
+              'appmagic-label-single-line': !properties.Wrap()
+            },
+            attr: {
+              'aria-live': live,
+              'aria-atomic': live() ? 'true' : null
+            }
+          }"&gt; con selettore ["#fullscreen-app-host","div[data-shortcut-id=\"989\"] &gt; .appmagic-label-text[unselectable=\"off\"][spellcheck=\"false\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/d55b30cf-4a1e-4e91-a788-cfd7958f9ad4_x000D_
 _x000D_
 Possibile Metodologia Risolutiva:_x000D_
-001 - Assegna a ogni pulsante un nome accessibile utilizzando il contenuto visibile (es. testo) o attributi come aria-label o aria-labelledby. Ad esempio: &lt;button aria-label="Invia"&gt;._x000D_
+001 - Aumenta il contrasto tra testo e sfondo per rendere il contenuto leggibile da utenti con difficoltà visive. WCAG richiede un rapporto di almeno 4.5:1 per il testo normale e 3:1 per il testo grande, quindi scegli colori che rispettino queste soglie._x000D_
 _x000D_
 Occorrenze rilevate: 1_x000D_
 _x000D_
@@ -845,26 +948,326 @@
 </t>
   </si>
   <si>
-    <t>..SITO_RUO_SERVIZIPERTE_202509 ** FARE SETUP SILK AP/PK - INBOX - SERVIZI / EP **</t>
-  </si>
-  <si>
-    <t>S001 prova</t>
-  </si>
-  <si>
-    <t>S001 homepage</t>
-  </si>
-  <si>
-    <t>serviziPerTe - 9.1.1.1 Contenuti non testuali - S001 homepage:</t>
-  </si>
-  <si>
-    <t>serviziPerTe - 9.4.1.2 Contenuti non testuali - S002 homepage:</t>
-  </si>
-  <si>
-    <t>serviziPerTe - 9.1.1.1 Contenuti non testuali - S001 homepage:: (#D000… descrizione)</t>
-  </si>
-  <si>
-    <t>serviziPerTe - 9.4.1.2 Nome, ruolo, valore - S001 homepage:: (#D0023)
-02 homepage:: (#D000… descrizione)</t>
+    <t xml:space="preserve">RUO - Insieme - 9.2.1.1 Tastiera - S001 Raccolta Idee e Contributi:: (#TM0009)_x000D_
+S001 Raccolta Idee e Contributi_x000D_
+Requisito WCAG: 2.1.1_x000D_
+Disabilità afflitte: Blind;Deafblind;Mobility_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - L'area scorrevole deve avere accesso da tastiera - Assicurarsi che gli elementi con contenuto scorrevole siano accessibili tramite tastiera [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.7/scrollable-region-focusable?application=playwright)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div class="virtualized-gallery" aria-label="Raccolta" role="list" data-control-part="gallery-window" style="position: absolute; inset: 0px; overflow: hidden auto;"&gt; con selettore ["#fullscreen-app-host","div[data-pa-item-id=\"344\"] &gt; .appmagic-borderfill-container &gt; .appmagic-border-inner &gt; .container_w3lqqm.accessibility-container &gt; .appmagic-gallery.vertical &gt; .virtualized-gallery[aria-label=\"Raccolta\"][role=\"list\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/01012ddd-657d-461c-80b5-c207b1827f41_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - L'elemento dovrebbe avere contenuto focalizzabile.
+L'elemento dovrebbe essere focalizzabile._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.2.4.2 Titolazione della pagina - S001 Raccolta Idee e Contributi:: (#TM0003)_x000D_
+S001 Raccolta Idee e Contributi_x000D_
+Requisito WCAG: 2.4.2_x000D_
+Disabilità afflitte: Blind;Deafblind_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - Il &lt;title&gt; della pagina non identifica lo scopo della pagina - L'elemento &lt;title&gt; di questa pagina non identifica il contenuto o lo scopo della pagina. [Ulteriori informazioni] (https://docs.deque.com/issue-help/1.0.0/en/title-not-meaningful)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;title&gt;INSIEME - Collaudo - Power Apps&lt;/title&gt; con selettore ["title"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/62cf55ae-54ae-4265-947e-fe6996c273d2_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - il &lt;title&gt; della pagina DEVE essere accurato e informativo. Il &lt;title&gt; della pagina DOVREBBE essere unico, se possibile.
+Le persone non vedenti non possono esaminare visivamente una pagina per identificare rapidamente il suo scopo. L'elemento &lt;title&gt; è la prima cosa letta da un lettore di schermo quando si carica una pagina o si passa a una nuova scheda del browser. Un &lt;title&gt; descrittivo offre agli utenti un rapido riepilogo della pagina senza doverla leggere completamente._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.3.1.2 Parti in lingua - S001 Raccolta Idee e Contributi:: (#TM0012)_x000D_
+S001 Raccolta Idee e Contributi_x000D_
+Requisito WCAG: 3.1.2_x000D_
+Disabilità afflitte: Blind;Cognitive;Deafblind_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - Gli attributi '[lang]' non hanno un valore valido - La specifica di una [lingua BCP 47] (https://www.w3.org/International/questions/qa-choosing-language-tags#question) valida per gli elementi consente di garantire che il testo venga pronunciato correttamente da uno screen reader. [Ulteriori informazioni] (https://web.dev/valid-lang/)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div class="appmagic-content-control-name appmagic-control-view canvasContentDiv _vst_" lang="271,5" data-control-id="734" data-control-name="Checkbox2_2" style="position: absolute; top: 191px; left: 271.5px; width: 150px; height: 50px; z-index: 22;"&gt; con selettore ["#fullscreen-app-host","div[data-control-id=\"734\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/b0b5fe6a-272b-439f-8c23-fc57e93c14de_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - Imposta un attributo lang valido sull’&lt;html&gt;._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.4.1.2 Nome, ruolo, valore - S001 Raccolta Idee e Contributi:: (#TM0004)_x000D_
+S001 Raccolta Idee e Contributi_x000D_
+Requisito WCAG: 4.1.2_x000D_
+Disabilità afflitte: Blind;Deafblind;Mobility_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - I campi di attivazione/disattivazione ARIA devono avere un nome accessibile - Assicurarsi che ogni campo di attivazione/disattivazione ARIA abbia un nome accessibile [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.8/aria-toggle-field-name?application=playwright)_x000D_
+002 - I pulsanti non hanno un nome accessibile - Quando un pulsante non ha un nome accessibile, le utilità per la lettura dello schermo lo annunciano come "pulsante", rendendolo inutilizzabile per gli utenti che si affidano alle utilità per la lettura dello schermo. [Ulteriori informazioni] (https://web.dev/button-name/)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div class="appmagic-toggleSwitch no-focus-outline left" role="switch" data-bind="{
+            style: {
+              height: AppMagic.Controls.converters.pxVerticalConverter.view(toggleHeight),
+              width: AppMagic.Controls.converters.pxHorizontalConverter.view(toggleWidth),
+              borderRadius: AppMagic.Controls.converters.pxVerticalConverter.view(toggleHeight / 2),
+            },
+            attr: {
+              title: properties.Tooltip() || null,
+              'aria-label': properties.AccessibleLabel() || null,
+              'aria-describedby': properties.ShowLabel() ? labelId : null,
+              'aria-checked': properties.Value() ? 'true' : 'false',
+              'aria-disabled': viewState.displayMode() !== AppMagic.Constants.DisplayMode.Edit
+            },
+            disable: viewState.displayMode() === AppMagic.Constants.DisplayMode.Disabled || viewState.displayMode() === AppMagic.Constants.DisplayMode.View,
+            shortcut: {
+              provider: shortcutProvider
+            },
+            css: {
+              disabled: viewState.displayMode() === AppMagic.Constants.DisplayMode.Disabled,
+              readonly: viewState.displayMode() === AppMagic.Constants.DisplayMode.View,
+              left: properties.TextPosition() === 'right',
+              right: properties.TextPosition() === 'left'
+            },
+            visible: viewState.displayMode() !== AppMagic.Constants.DisplayMode.View
+          }" aria-describedby="toggleSwitch_siena_5165c789384250_label" aria-checked="false" data-shortcut-id="140" tabindex="65" style="height: 28px; width: 52px; border-radius: 14px;"&gt; con selettore ["#fullscreen-app-host","div[data-shortcut-id=\"140\"]"]_x000D_
+002 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;button class="appmagic-button-container no-focus-outline" data-control-part="button" data-bind="
+      event: {
+        click: handleClick,
+        pointerdown: handleMouseDown,
+        pointerup: handleMouseUp,
+        pointerout: handleMouseOut
+      },
+      attr: {
+        title: properties.Tooltip,
+        disabled: viewState.displayMode() !== AppMagic.Constants.DisplayMode.Edit
+      }
+    " title="" tabindex="76"&gt; con selettore ["#fullscreen-app-host","div[data-control-id=\"658\"] &gt; .appmagic-borderfill-container &gt; .appmagic-border-inner &gt; .react-knockout-control &gt; .appmagic-button-wrapper &gt; .appmagic-button-container[data-control-part=\"button\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/603533ef-362a-4ecb-9c51-32e6f4921c04_x000D_
+002 - https://axe.deque.com/issues/a57011c9-2c02-4a44-b63a-55b77949f89d_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - Usa aria-pressed (true/false) con role="button" o direttamente &lt;button&gt;._x000D_
+002 - Assegna a ogni pulsante un nome accessibile utilizzando il contenuto visibile (es. testo) o attributi come aria-label o aria-labelledby. Ad esempio: &lt;button aria-label="Invia"&gt;._x000D_
+_x000D_
+Occorrenze rilevate: 2_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.1.4.3 Contrasto (minimo) - S002 Composizione dei Team:: (#TM0036)_x000D_
+S002 Composizione dei Team_x000D_
+Requisito WCAG: 1.4.3_x000D_
+Disabilità afflitte: Colorblindness;Low Vision_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - I colori di sfondo e di primo piano non hanno un rapporto di contrasto sufficiente. - Il testo a basso contrasto è difficile o impossibile da leggere per molti utenti. [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.10/color-contrast)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div spellcheck="false" unselectable="off" class="appmagic-label-text" data-control-part="text" data-bind="{
+            inlineEditText: properties.Text,
+            css: {
+              'appmagic-label-single-line': !properties.Wrap()
+            },
+            attr: {
+              'aria-live': live,
+              'aria-atomic': live() ? 'true' : null
+            }
+          }"&gt; con selettore ["#fullscreen-app-host","div[title=\"cla3tum@posteitaliane.it\"] &gt; .appmagic-label-text[unselectable=\"off\"][spellcheck=\"false\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/0d607325-a0de-4c58-b38f-f63846d79714_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - Aumenta il contrasto tra testo e sfondo per rendere il contenuto leggibile da utenti con difficoltà visive. WCAG richiede un rapporto di almeno 4.5:1 per il testo normale e 3:1 per il testo grande, quindi scegli colori che rispettino queste soglie._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.2.1.1 Tastiera - S002 Composizione dei Team:: (#TM0046)_x000D_
+S002 Composizione dei Team_x000D_
+Requisito WCAG: 2.1.1_x000D_
+Disabilità afflitte: Blind;Deafblind;Mobility_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - L'area scorrevole deve avere accesso da tastiera - Assicurarsi che gli elementi con contenuto scorrevole siano accessibili tramite tastiera [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.7/scrollable-region-focusable?application=playwright)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div class="virtualized-gallery" aria-label="Raccolta" role="list" data-control-part="gallery-window" style="position: absolute; inset: 0px; overflow: hidden auto;"&gt; con selettore ["#fullscreen-app-host","div[data-pa-item-id=\"156\"] &gt; .appmagic-borderfill-container &gt; .appmagic-border-inner &gt; .container_w3lqqm.accessibility-container &gt; .appmagic-gallery.vertical &gt; .virtualized-gallery[aria-label=\"Raccolta\"][role=\"list\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/49755aaa-05c4-4e62-bb23-62ee8537c745_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - L'elemento dovrebbe avere contenuto focalizzabile.
+L'elemento dovrebbe essere focalizzabile._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.2.4.2 Titolazione della pagina - S002 Composizione dei Team:: (#TM0039)_x000D_
+S002 Composizione dei Team_x000D_
+Requisito WCAG: 2.4.2_x000D_
+Disabilità afflitte: Blind;Deafblind_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - Il &lt;title&gt; della pagina non identifica lo scopo della pagina - L'elemento &lt;title&gt; di questa pagina non identifica il contenuto o lo scopo della pagina. [Ulteriori informazioni] (https://docs.deque.com/issue-help/1.0.0/en/title-not-meaningful)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;title&gt;INSIEME - Collaudo - Power Apps&lt;/title&gt; con selettore ["title"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/758e591f-4898-4554-ba57-a225c2a5c18b_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - il &lt;title&gt; della pagina DEVE essere accurato e informativo. Il &lt;title&gt; della pagina DOVREBBE essere unico, se possibile.
+Le persone non vedenti non possono esaminare visivamente una pagina per identificare rapidamente il suo scopo. L'elemento &lt;title&gt; è la prima cosa letta da un lettore di schermo quando si carica una pagina o si passa a una nuova scheda del browser. Un &lt;title&gt; descrittivo offre agli utenti un rapido riepilogo della pagina senza doverla leggere completamente._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.3.1.1 Lingua della pagina - S002 Composizione dei Team:: (#TM0038)_x000D_
+S002 Composizione dei Team_x000D_
+Requisito WCAG: 3.1.1_x000D_
+Disabilità afflitte: Blind;Cognitive;Deafblind_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - L'attributo Lang per la pagina non è la lingua principale della pagina - Il valore dell'attributo lang utilizzato per indicare la lingua principale della pagina è per la lingua errata. [Ulteriori informazioni] (https://docs.deque.com/issue-help/1.0.0/en/lang-not-accurate)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506  con selettore ["html"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/a27720be-c162-486f-8bdc-5bdcf309c62a_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - Assicurarsi che l'attributo lang specificato nell'elemento &lt;html&gt; corrisponda correttamente alla lingua principale del contenuto della pagina. Ad esempio, per indicare l'italiano come lingua principale, utilizzare &lt;html lang="it"&gt;. Verificare la correttezza del valore con strumenti di validazione e aggiornare eventuali errori._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUO - Insieme - 9.4.1.2 Nome, ruolo, valore - S002 Composizione dei Team:: (#TM0040)_x000D_
+S002 Composizione dei Team_x000D_
+Requisito WCAG: 4.1.2_x000D_
+Disabilità afflitte: Blind;Deafblind;Mobility_x000D_
+Impatto Utente: 2 - Serious_x000D_
+_x000D_
+Descrizione_x000D_
+001 - I campi di attivazione/disattivazione ARIA devono avere un nome accessibile - Assicurarsi che ogni campo di attivazione/disattivazione ARIA abbia un nome accessibile [Ulteriori informazioni] (https://dequeuniversity.com/rules/axe/4.8/aria-toggle-field-name?application=playwright)_x000D_
+_x000D_
+Esempio di violazione individuata sull'oggetto:_x000D_
+001 - https://apps.powerapps.com/play/e/default-761de76f-3d5c-4174-917c-5ad4d06360cb/a/6891c1e8-c00a-4655-bdd3-e5349671a051?tenantId=761de76f-3d5c-4174-917c-5ad4d06360cb&amp;hint=6db5d4d8-79d5-4cb9-ab21-16e940158554&amp;sourcetime=1754387821506 &lt;div class="appmagic-toggleSwitch no-focus-outline right" role="switch" data-bind="{
+            style: {
+              height: AppMagic.Controls.converters.pxVerticalConverter.view(toggleHeight),
+              width: AppMagic.Controls.converters.pxHorizontalConverter.view(toggleWidth),
+              borderRadius: AppMagic.Controls.converters.pxVerticalConverter.view(toggleHeight / 2),
+            },
+            attr: {
+              title: properties.Tooltip() || null,
+              'aria-label': properties.AccessibleLabel() || null,
+              'aria-describedby': properties.ShowLabel() ? labelId : null,
+              'aria-checked': properties.Value() ? 'true' : 'false',
+              'aria-disabled': viewState.displayMode() !== AppMagic.Constants.DisplayMode.Edit
+            },
+            disable: viewState.displayMode() === AppMagic.Constants.DisplayMode.Disabled || viewState.displayMode() === AppMagic.Constants.DisplayMode.View,
+            shortcut: {
+              provider: shortcutProvider
+            },
+            css: {
+              disabled: viewState.displayMode() === AppMagic.Constants.DisplayMode.Disabled,
+              readonly: viewState.displayMode() === AppMagic.Constants.DisplayMode.View,
+              left: properties.TextPosition() === 'right',
+              right: properties.TextPosition() === 'left'
+            },
+            visible: viewState.displayMode() !== AppMagic.Constants.DisplayMode.View
+          }" aria-describedby="toggleSwitch_siena_3c3e540276aae38_label" aria-checked="false" data-shortcut-id="84" tabindex="96" style="height: 30px; width: 55px; border-radius: 15px;"&gt; con selettore ["#fullscreen-app-host","div[data-shortcut-id=\"84\"]"]_x000D_
+_x000D_
+Dettaglio + screenshot (accedere con le seguenti credenziali: user, axeposte@gmail.com; password, Poste2024!)_x000D_
+001 - https://axe.deque.com/issues/9b9a718e-0768-4125-aafa-520c95d78b65_x000D_
+_x000D_
+Possibile Metodologia Risolutiva:_x000D_
+001 - Usa aria-pressed (true/false) con role="button" o direttamente &lt;button&gt;._x000D_
+_x000D_
+Occorrenze rilevate: 1_x000D_
+_x000D_
+Link al dettaglio requisito WCAG: https://www.w3.org/WAI/WCAG21/quickref/_x000D_
+</t>
+  </si>
+  <si>
+    <t>S001 Raccolta Idee e Contributi</t>
+  </si>
+  <si>
+    <t>S002 Composizione dei Team</t>
+  </si>
+  <si>
+    <t>9.1.3.1</t>
+  </si>
+  <si>
+    <t>9.1.4.3</t>
+  </si>
+  <si>
+    <t>9.2.1.1</t>
+  </si>
+  <si>
+    <t>9.2.4.2</t>
+  </si>
+  <si>
+    <t>9.3.1.2</t>
+  </si>
+  <si>
+    <t>9.3.1.1</t>
+  </si>
+  <si>
+    <t>AP-00000</t>
+  </si>
+  <si>
+    <t>RUO_INSIEME</t>
   </si>
 </sst>
 </file>
@@ -986,7 +1389,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1001,7 +1404,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calcolo" xfId="1" builtinId="22"/>
@@ -1018,6 +1420,34 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="load to silk"/>
+      <sheetName val="Copertina"/>
+      <sheetName val="Page Status_Summary"/>
+      <sheetName val="Pivot"/>
+      <sheetName val="Not Passed"/>
+      <sheetName val="InLab Test"/>
+      <sheetName val="Dati input"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2152,10 +2582,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1351EE81-E912-4391-8C73-E5B6D3C40707}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.6640625" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
@@ -2195,56 +2626,310 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.1.3.1 Informazioni e correlazioni - S001 Raccolta Idee e Contributi:</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>36</v>
+        <v>164</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" t="s">
-        <v>139</v>
+      <c r="I2" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.1.4.3 Contrasto (minimo) - S001 Raccolta Idee e Contributi:</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.2.1.1 Tastiera - S001 Raccolta Idee e Contributi:</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" s="5" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.2.4.2 Titolazione della pagina - S001 Raccolta Idee e Contributi:</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.3.1.2 Parti in lingua - S001 Raccolta Idee e Contributi:</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="5" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.4.1.2 Nome, ruolo, valore - S001 Raccolta Idee e Contributi:</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="H3" s="5"/>
-      <c r="I3" t="s">
-        <v>139</v>
+      <c r="G7" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.1.4.3 Contrasto (minimo) - S002 Composizione dei Team:</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="5" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.2.1.1 Tastiera - S002 Composizione dei Team:</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.2.4.2 Titolazione della pagina - S002 Composizione dei Team:</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="5" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.3.1.1 Lingua della pagina - S002 Composizione dei Team:</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <f>_xlfn.XLOOKUP([1]!outTable[[#This Row],[ID Silk]],[1]!Tabella4[ID Silk],[1]!Tabella4[Titolo Defect],,0,1)</f>
+        <v>RUO - Insieme - 9.4.1.2 Nome, ruolo, valore - S002 Composizione dei Team:</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -2299,53 +2984,53 @@
         <v>132</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>145</v>
+        <v>138</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>51</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>